<commit_message>
update file test-case setelah eksekusi
</commit_message>
<xml_diff>
--- a/test-cases/Test_Cases_SauceDemo.xlsx
+++ b/test-cases/Test_Cases_SauceDemo.xlsx
@@ -8,24 +8,33 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FASILKOM\MySkill\SAUCEDEMO\manual-qa-saucedemo\test-cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FA50983-0E89-4C1B-BAD3-54ADC4DBCC37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD2ACB05-202E-4BD9-9B45-29610C14B020}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1900" yWindow="1660" windowWidth="13780" windowHeight="9140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="243">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -100,9 +109,6 @@
     <t>User is redirected to the inventory page and product list is displayed.</t>
   </si>
   <si>
-    <t>Not Executed</t>
-  </si>
-  <si>
     <t>TC-AUTH-002</t>
   </si>
   <si>
@@ -623,9 +629,6 @@
     <t>User is on checkout complete page.</t>
   </si>
   <si>
-    <t>1. Click Back Home.</t>
-  </si>
-  <si>
     <t>Checkout complete page opened</t>
   </si>
   <si>
@@ -702,13 +705,141 @@
   </si>
   <si>
     <t>Button label changes from Add to cart to Remove for the selected product.</t>
+  </si>
+  <si>
+    <t>User successfully logged in and was redirected to the inventory page displaying the product list</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>The inventory page successfully displays a list of available products.</t>
+  </si>
+  <si>
+    <t>The selected product is successfully added to the cart and the cart icon increases by 1.</t>
+  </si>
+  <si>
+    <t>The selected item is successfully removed from the cart list and the cart icon is successfully updated.</t>
+  </si>
+  <si>
+    <t>The user was successfully redirected to the payment information page.</t>
+  </si>
+  <si>
+    <t>The user is successfully redirected to the payment process summary page.</t>
+  </si>
+  <si>
+    <t>The overview page successfully displays an accurate order summary and calculated total.</t>
+  </si>
+  <si>
+    <t>The order has been completed and the confirmation page is successfully displayed.</t>
+  </si>
+  <si>
+    <t>The user was successfully logged out of the account and redirected to the login page.</t>
+  </si>
+  <si>
+    <t>The page successfully displays each product card with an image, title, description, price, and action button.</t>
+  </si>
+  <si>
+    <t>Products are successfully sorted alphabetically from A to Z.</t>
+  </si>
+  <si>
+    <t>Products have been successfully sorted from lowest to highest price.</t>
+  </si>
+  <si>
+    <t>The selected product's detail page has opened with matching information.</t>
+  </si>
+  <si>
+    <t>User successfully returned to the inventory page.</t>
+  </si>
+  <si>
+    <t>The shopping cart page opens and successfully displays the same items as those selected.</t>
+  </si>
+  <si>
+    <t>The product is successfully removed from the cart and the cart badge is updated.</t>
+  </si>
+  <si>
+    <t>All selected products are successfully added and the cart badge displays the correct total amount.</t>
+  </si>
+  <si>
+    <t>1. Click Continue Shopping</t>
+  </si>
+  <si>
+    <t>The system successfully displays an error message and the user remains on the login page.</t>
+  </si>
+  <si>
+    <t>The system successfully displays an error message stating that the username field is required.</t>
+  </si>
+  <si>
+    <t>The system successfully displays an error message stating that the password field is required.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">System displayed the error message </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>“Username is required”</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and did not allow the user to log in.</t>
+    </r>
+  </si>
+  <si>
+    <t>The system successfully displayed a validation error due to a missing First Name.</t>
+  </si>
+  <si>
+    <t>The system successfully displayed a validation error due to a missing Last Name.</t>
+  </si>
+  <si>
+    <t>The system successfully displayed a validation error due to a missing Zip Code.</t>
+  </si>
+  <si>
+    <t>The user successfully returned to the shopping cart page without completing the payment process.</t>
+  </si>
+  <si>
+    <t>Validation worked as expected when both username and password were left empty. The system prioritized the username validation message.</t>
+  </si>
+  <si>
+    <t>UI issue found on the login error message display. Message visibility/readability is inconsistent depending on window size.</t>
+  </si>
+  <si>
+    <t>Error message was visible, but part of the text was clipped at the default window size. The full message was only readable after resizing the browser window smaller.</t>
+  </si>
+  <si>
+    <t>The button label has successfully changed from “Add to cart” to “Remove” for the selected product.</t>
+  </si>
+  <si>
+    <t>The cart badge is successfully visible in the correct amount across the page.</t>
+  </si>
+  <si>
+    <t>The cart icon is visible and successfully opens the cart page when clicked.</t>
+  </si>
+  <si>
+    <t>Fail</t>
+  </si>
+  <si>
+    <t>None</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -722,6 +853,14 @@
       <color rgb="FF1F1F1F"/>
       <name val="Carlito"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -731,7 +870,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -808,17 +947,6 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FFD0D7DE"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FFD0D7DE"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -849,8 +977,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1141,8 +1269,8 @@
     <col min="4" max="4" width="37.08984375" customWidth="1"/>
     <col min="5" max="5" width="13.08984375" customWidth="1"/>
     <col min="6" max="6" width="16.36328125" customWidth="1"/>
-    <col min="7" max="7" width="26.1796875" customWidth="1"/>
-    <col min="8" max="8" width="39.26953125" customWidth="1"/>
+    <col min="7" max="7" width="35.36328125" customWidth="1"/>
+    <col min="8" max="8" width="52" customWidth="1"/>
     <col min="9" max="9" width="26.1796875" customWidth="1"/>
     <col min="10" max="10" width="37.08984375" customWidth="1"/>
     <col min="11" max="11" width="24" customWidth="1"/>
@@ -1222,209 +1350,233 @@
       <c r="J2" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="K2" s="5"/>
-      <c r="L2" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M2" s="6"/>
+      <c r="K2" s="9" t="s">
+        <v>208</v>
+      </c>
+      <c r="L2" t="s">
+        <v>209</v>
+      </c>
+      <c r="M2" s="6" t="s">
+        <v>242</v>
+      </c>
     </row>
     <row r="3" spans="1:13" ht="22.65" customHeight="1">
       <c r="A3" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C3" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" s="5" t="s">
         <v>25</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>26</v>
       </c>
       <c r="E3" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G3" s="5" t="s">
         <v>19</v>
       </c>
       <c r="H3" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="I3" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="J3" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="J3" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="K3" s="5"/>
-      <c r="L3" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M3" s="6"/>
+      <c r="K3" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="L3" t="s">
+        <v>209</v>
+      </c>
+      <c r="M3" s="6" t="s">
+        <v>242</v>
+      </c>
     </row>
     <row r="4" spans="1:13" ht="22.65" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C4" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D4" s="5" t="s">
         <v>32</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>33</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G4" s="5" t="s">
         <v>19</v>
       </c>
       <c r="H4" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="I4" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="I4" s="5" t="s">
+      <c r="J4" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="J4" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="K4" s="5"/>
-      <c r="L4" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M4" s="6"/>
+      <c r="K4" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="L4" t="s">
+        <v>209</v>
+      </c>
+      <c r="M4" s="6" t="s">
+        <v>242</v>
+      </c>
     </row>
     <row r="5" spans="1:13" ht="22.65" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C5" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D5" s="5" t="s">
         <v>38</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>39</v>
       </c>
       <c r="E5" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G5" s="5" t="s">
         <v>19</v>
       </c>
       <c r="H5" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="I5" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="I5" s="5" t="s">
+      <c r="J5" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="J5" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="K5" s="5"/>
-      <c r="L5" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M5" s="6"/>
+      <c r="K5" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="L5" t="s">
+        <v>209</v>
+      </c>
+      <c r="M5" s="6" t="s">
+        <v>242</v>
+      </c>
     </row>
     <row r="6" spans="1:13" ht="22.65" customHeight="1">
       <c r="A6" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C6" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D6" s="5" t="s">
         <v>44</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>45</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G6" s="5" t="s">
         <v>19</v>
       </c>
       <c r="H6" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="I6" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="I6" s="5" t="s">
+      <c r="J6" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="J6" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="K6" s="5"/>
-      <c r="L6" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M6" s="6"/>
+      <c r="K6" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="L6" t="s">
+        <v>209</v>
+      </c>
+      <c r="M6" s="5" t="s">
+        <v>235</v>
+      </c>
     </row>
     <row r="7" spans="1:13" ht="22.65" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C7" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="E7" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="F7" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="F7" s="5" t="s">
+      <c r="G7" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="G7" s="5" t="s">
+      <c r="H7" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="H7" s="5" t="s">
+      <c r="I7" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="I7" s="5" t="s">
+      <c r="J7" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="J7" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="K7" s="5"/>
-      <c r="L7" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M7" s="6"/>
+      <c r="K7" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="L7" t="s">
+        <v>209</v>
+      </c>
+      <c r="M7" s="6" t="s">
+        <v>242</v>
+      </c>
     </row>
     <row r="8" spans="1:13" ht="22.65" customHeight="1">
       <c r="A8" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="C8" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="D8" s="5" t="s">
         <v>60</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>61</v>
       </c>
       <c r="E8" s="5" t="s">
         <v>17</v>
@@ -1433,220 +1585,244 @@
         <v>18</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H8" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="J8" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="I8" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="J8" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="K8" s="5"/>
-      <c r="L8" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M8" s="6"/>
+      <c r="K8" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="L8" t="s">
+        <v>209</v>
+      </c>
+      <c r="M8" s="6" t="s">
+        <v>242</v>
+      </c>
     </row>
     <row r="9" spans="1:13" ht="22.65" customHeight="1">
       <c r="A9" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="B9" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="C9" s="5" t="s">
+      <c r="D9" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="E9" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G9" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="E9" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="G9" s="5" t="s">
+      <c r="H9" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="H9" s="5" t="s">
+      <c r="I9" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="I9" s="5" t="s">
+      <c r="J9" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="J9" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="K9" s="5"/>
-      <c r="L9" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M9" s="6"/>
+      <c r="K9" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="L9" t="s">
+        <v>209</v>
+      </c>
+      <c r="M9" s="6" t="s">
+        <v>242</v>
+      </c>
     </row>
     <row r="10" spans="1:13" ht="22.65" customHeight="1">
       <c r="A10" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="B10" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="C10" s="5" t="s">
+      <c r="D10" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="E10" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="H10" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="E10" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="G10" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="H10" s="5" t="s">
+      <c r="I10" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="J10" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="I10" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="J10" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="K10" s="5"/>
-      <c r="L10" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M10" s="6"/>
+      <c r="K10" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="L10" t="s">
+        <v>209</v>
+      </c>
+      <c r="M10" s="6" t="s">
+        <v>242</v>
+      </c>
     </row>
     <row r="11" spans="1:13" ht="22.65" customHeight="1">
       <c r="A11" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="B11" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="C11" s="5" t="s">
+      <c r="D11" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="E11" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="H11" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="E11" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="G11" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="H11" s="5" t="s">
+      <c r="I11" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="J11" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="I11" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="J11" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="K11" s="5"/>
-      <c r="L11" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M11" s="6"/>
+      <c r="K11" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="L11" t="s">
+        <v>209</v>
+      </c>
+      <c r="M11" s="6" t="s">
+        <v>242</v>
+      </c>
     </row>
     <row r="12" spans="1:13" ht="22.65" customHeight="1">
       <c r="A12" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="C12" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="B12" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="C12" s="5" t="s">
+      <c r="D12" s="5" t="s">
         <v>82</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>83</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H12" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="I12" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="J12" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="I12" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="J12" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="K12" s="5"/>
-      <c r="L12" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M12" s="6"/>
+      <c r="K12" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="L12" t="s">
+        <v>209</v>
+      </c>
+      <c r="M12" s="6" t="s">
+        <v>242</v>
+      </c>
     </row>
     <row r="13" spans="1:13" ht="22.65" customHeight="1">
       <c r="A13" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="C13" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="B13" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="C13" s="5" t="s">
+      <c r="D13" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="E13" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="E13" s="5" t="s">
+      <c r="F13" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G13" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="F13" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="G13" s="5" t="s">
+      <c r="H13" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="H13" s="5" t="s">
+      <c r="I13" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="I13" s="5" t="s">
+      <c r="J13" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="J13" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="K13" s="5"/>
-      <c r="L13" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M13" s="6"/>
+      <c r="K13" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="L13" t="s">
+        <v>209</v>
+      </c>
+      <c r="M13" s="6" t="s">
+        <v>242</v>
+      </c>
     </row>
     <row r="14" spans="1:13" ht="22.65" customHeight="1">
       <c r="A14" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B14" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="C14" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="D14" s="5" t="s">
         <v>96</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>97</v>
       </c>
       <c r="E14" s="5" t="s">
         <v>17</v>
@@ -1655,220 +1831,244 @@
         <v>18</v>
       </c>
       <c r="G14" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="H14" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="H14" s="5" t="s">
+      <c r="I14" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="J14" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="I14" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="J14" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="K14" s="5"/>
-      <c r="L14" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M14" s="6"/>
+      <c r="K14" s="5" t="s">
+        <v>211</v>
+      </c>
+      <c r="L14" t="s">
+        <v>209</v>
+      </c>
+      <c r="M14" s="6" t="s">
+        <v>242</v>
+      </c>
     </row>
     <row r="15" spans="1:13" ht="22.65" customHeight="1">
       <c r="A15" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C15" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="B15" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="C15" s="5" t="s">
+      <c r="D15" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="D15" s="5" t="s">
+      <c r="E15" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G15" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="E15" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="F15" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="G15" s="5" t="s">
+      <c r="H15" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="H15" s="5" t="s">
+      <c r="I15" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="I15" s="5" t="s">
+      <c r="J15" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="J15" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="K15" s="5"/>
-      <c r="L15" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M15" s="6"/>
+      <c r="K15" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="L15" t="s">
+        <v>209</v>
+      </c>
+      <c r="M15" s="6" t="s">
+        <v>242</v>
+      </c>
     </row>
     <row r="16" spans="1:13" ht="22.65" customHeight="1">
       <c r="A16" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C16" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="B16" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="C16" s="5" t="s">
+      <c r="D16" s="5" t="s">
         <v>109</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>110</v>
       </c>
       <c r="E16" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H16" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="I16" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="J16" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="I16" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="J16" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="K16" s="5"/>
-      <c r="L16" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M16" s="6"/>
+      <c r="K16" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="L16" t="s">
+        <v>209</v>
+      </c>
+      <c r="M16" s="6" t="s">
+        <v>242</v>
+      </c>
     </row>
     <row r="17" spans="1:13" ht="22.65" customHeight="1">
       <c r="A17" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C17" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="B17" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="C17" s="5" t="s">
+      <c r="D17" s="5" t="s">
         <v>114</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>115</v>
       </c>
       <c r="E17" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G17" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="H17" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="H17" s="5" t="s">
+      <c r="I17" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="I17" s="5" t="s">
+      <c r="J17" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="J17" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="K17" s="5"/>
-      <c r="L17" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M17" s="6"/>
+      <c r="K17" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="L17" t="s">
+        <v>209</v>
+      </c>
+      <c r="M17" s="6" t="s">
+        <v>242</v>
+      </c>
     </row>
     <row r="18" spans="1:13" ht="22.65" customHeight="1">
       <c r="A18" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C18" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="B18" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="C18" s="5" t="s">
+      <c r="D18" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="D18" s="5" t="s">
+      <c r="E18" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G18" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="E18" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="F18" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="G18" s="5" t="s">
+      <c r="H18" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="H18" s="5" t="s">
+      <c r="I18" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="I18" s="5" t="s">
+      <c r="J18" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="J18" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="K18" s="5"/>
-      <c r="L18" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M18" s="6"/>
+      <c r="K18" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="L18" t="s">
+        <v>209</v>
+      </c>
+      <c r="M18" s="6" t="s">
+        <v>242</v>
+      </c>
     </row>
     <row r="19" spans="1:13" ht="22.65" customHeight="1">
       <c r="A19" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C19" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="B19" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="C19" s="5" t="s">
+      <c r="D19" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="D19" s="5" t="s">
+      <c r="E19" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="F19" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="E19" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="F19" s="5" t="s">
+      <c r="G19" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="G19" s="5" t="s">
+      <c r="H19" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="H19" s="5" t="s">
+      <c r="I19" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="I19" s="5" t="s">
+      <c r="J19" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="J19" s="5" t="s">
-        <v>134</v>
-      </c>
-      <c r="K19" s="5"/>
-      <c r="L19" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M19" s="6"/>
+      <c r="K19" s="5" t="s">
+        <v>239</v>
+      </c>
+      <c r="L19" t="s">
+        <v>209</v>
+      </c>
+      <c r="M19" s="6" t="s">
+        <v>242</v>
+      </c>
     </row>
     <row r="20" spans="1:13" ht="22.65" customHeight="1">
       <c r="A20" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="B20" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="C20" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="C20" s="5" t="s">
+      <c r="D20" s="5" t="s">
         <v>137</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>138</v>
       </c>
       <c r="E20" s="5" t="s">
         <v>17</v>
@@ -1877,220 +2077,244 @@
         <v>18</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H20" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="I20" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="I20" s="5" t="s">
+      <c r="J20" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="J20" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="K20" s="5"/>
-      <c r="L20" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M20" s="6"/>
+      <c r="K20" s="5" t="s">
+        <v>213</v>
+      </c>
+      <c r="L20" t="s">
+        <v>209</v>
+      </c>
+      <c r="M20" s="6" t="s">
+        <v>242</v>
+      </c>
     </row>
     <row r="21" spans="1:13" ht="22.65" customHeight="1">
       <c r="A21" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="C21" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="B21" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="C21" s="5" t="s">
+      <c r="D21" s="5" t="s">
         <v>143</v>
-      </c>
-      <c r="D21" s="5" t="s">
-        <v>144</v>
       </c>
       <c r="E21" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G21" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="H21" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="H21" s="5" t="s">
+      <c r="I21" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="I21" s="5" t="s">
+      <c r="J21" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="J21" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="K21" s="5"/>
-      <c r="L21" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M21" s="6"/>
+      <c r="K21" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="L21" t="s">
+        <v>209</v>
+      </c>
+      <c r="M21" s="6" t="s">
+        <v>242</v>
+      </c>
     </row>
     <row r="22" spans="1:13" ht="22.65" customHeight="1">
       <c r="A22" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="C22" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="B22" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="C22" s="5" t="s">
+      <c r="D22" s="5" t="s">
         <v>150</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>151</v>
       </c>
       <c r="E22" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H22" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="I22" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="I22" s="5" t="s">
+      <c r="J22" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="J22" s="5" t="s">
-        <v>154</v>
-      </c>
-      <c r="K22" s="5"/>
-      <c r="L22" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M22" s="6"/>
+      <c r="K22" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="L22" t="s">
+        <v>209</v>
+      </c>
+      <c r="M22" s="6" t="s">
+        <v>242</v>
+      </c>
     </row>
     <row r="23" spans="1:13" ht="22.65" customHeight="1">
       <c r="A23" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="C23" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="B23" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="C23" s="5" t="s">
+      <c r="D23" s="5" t="s">
         <v>156</v>
-      </c>
-      <c r="D23" s="5" t="s">
-        <v>157</v>
       </c>
       <c r="E23" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H23" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="I23" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="I23" s="5" t="s">
+      <c r="J23" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="J23" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="K23" s="5"/>
-      <c r="L23" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M23" s="6"/>
+      <c r="K23" s="5" t="s">
+        <v>233</v>
+      </c>
+      <c r="L23" t="s">
+        <v>209</v>
+      </c>
+      <c r="M23" s="6" t="s">
+        <v>242</v>
+      </c>
     </row>
     <row r="24" spans="1:13" ht="22.65" customHeight="1">
       <c r="A24" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="C24" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="B24" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="C24" s="5" t="s">
+      <c r="D24" s="5" t="s">
         <v>162</v>
-      </c>
-      <c r="D24" s="5" t="s">
-        <v>163</v>
       </c>
       <c r="E24" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H24" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="I24" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="I24" s="5" t="s">
+      <c r="J24" s="5" t="s">
         <v>165</v>
       </c>
-      <c r="J24" s="5" t="s">
-        <v>166</v>
-      </c>
-      <c r="K24" s="5"/>
-      <c r="L24" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M24" s="6"/>
+      <c r="K24" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="L24" t="s">
+        <v>209</v>
+      </c>
+      <c r="M24" s="6" t="s">
+        <v>242</v>
+      </c>
     </row>
     <row r="25" spans="1:13" ht="22.65" customHeight="1">
       <c r="A25" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="C25" s="5" t="s">
         <v>167</v>
       </c>
-      <c r="B25" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="C25" s="5" t="s">
+      <c r="D25" s="5" t="s">
         <v>168</v>
-      </c>
-      <c r="D25" s="5" t="s">
-        <v>169</v>
       </c>
       <c r="E25" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G25" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="H25" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="H25" s="5" t="s">
+      <c r="I25" s="5" t="s">
         <v>171</v>
       </c>
-      <c r="I25" s="5" t="s">
+      <c r="J25" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="J25" s="5" t="s">
-        <v>173</v>
-      </c>
-      <c r="K25" s="5"/>
-      <c r="L25" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M25" s="6"/>
+      <c r="K25" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="L25" t="s">
+        <v>209</v>
+      </c>
+      <c r="M25" s="6" t="s">
+        <v>242</v>
+      </c>
     </row>
     <row r="26" spans="1:13" ht="22.65" customHeight="1">
       <c r="A26" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="C26" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="B26" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="C26" s="5" t="s">
+      <c r="D26" s="5" t="s">
         <v>175</v>
-      </c>
-      <c r="D26" s="5" t="s">
-        <v>176</v>
       </c>
       <c r="E26" s="5" t="s">
         <v>17</v>
@@ -2099,211 +2323,235 @@
         <v>18</v>
       </c>
       <c r="G26" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="H26" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="H26" s="5" t="s">
+      <c r="I26" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="J26" s="5" t="s">
         <v>178</v>
       </c>
-      <c r="I26" s="5" t="s">
-        <v>172</v>
-      </c>
-      <c r="J26" s="5" t="s">
-        <v>179</v>
-      </c>
-      <c r="K26" s="5"/>
-      <c r="L26" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M26" s="6"/>
+      <c r="K26" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="L26" t="s">
+        <v>209</v>
+      </c>
+      <c r="M26" s="6" t="s">
+        <v>242</v>
+      </c>
     </row>
     <row r="27" spans="1:13" ht="22.65" customHeight="1">
       <c r="A27" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="C27" s="5" t="s">
         <v>180</v>
       </c>
-      <c r="B27" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="C27" s="5" t="s">
+      <c r="D27" s="5" t="s">
         <v>181</v>
       </c>
-      <c r="D27" s="5" t="s">
+      <c r="E27" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="F27" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G27" s="5" t="s">
         <v>182</v>
       </c>
-      <c r="E27" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="F27" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="G27" s="5" t="s">
+      <c r="H27" s="5" t="s">
+        <v>226</v>
+      </c>
+      <c r="I27" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="H27" s="5" t="s">
-        <v>184</v>
-      </c>
-      <c r="I27" s="5" t="s">
-        <v>185</v>
-      </c>
       <c r="J27" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="K27" s="5"/>
-      <c r="L27" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M27" s="6"/>
+        <v>92</v>
+      </c>
+      <c r="K27" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="L27" t="s">
+        <v>209</v>
+      </c>
+      <c r="M27" s="6" t="s">
+        <v>242</v>
+      </c>
     </row>
     <row r="28" spans="1:13" ht="22.65" customHeight="1">
       <c r="A28" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="C28" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="B28" s="5" t="s">
+      <c r="D28" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="C28" s="5" t="s">
+      <c r="E28" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="F28" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="G28" s="5" t="s">
         <v>188</v>
       </c>
-      <c r="D28" s="5" t="s">
+      <c r="H28" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="E28" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="F28" s="5" t="s">
-        <v>187</v>
-      </c>
-      <c r="G28" s="5" t="s">
+      <c r="I28" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="J28" s="5" t="s">
         <v>190</v>
       </c>
-      <c r="H28" s="5" t="s">
-        <v>191</v>
-      </c>
-      <c r="I28" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="J28" s="5" t="s">
-        <v>192</v>
-      </c>
-      <c r="K28" s="5"/>
+      <c r="K28" s="5" t="s">
+        <v>237</v>
+      </c>
       <c r="L28" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M28" s="6"/>
+        <v>241</v>
+      </c>
+      <c r="M28" s="5" t="s">
+        <v>236</v>
+      </c>
     </row>
     <row r="29" spans="1:13" ht="22.65" customHeight="1">
       <c r="A29" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="D29" s="5" t="s">
         <v>193</v>
       </c>
-      <c r="B29" s="5" t="s">
-        <v>187</v>
-      </c>
-      <c r="C29" s="5" t="s">
+      <c r="E29" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="F29" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="G29" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="H29" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="D29" s="5" t="s">
+      <c r="I29" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="J29" s="5" t="s">
         <v>195</v>
       </c>
-      <c r="E29" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="F29" s="5" t="s">
-        <v>187</v>
-      </c>
-      <c r="G29" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="H29" s="5" t="s">
-        <v>196</v>
-      </c>
-      <c r="I29" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="J29" s="5" t="s">
-        <v>197</v>
-      </c>
-      <c r="K29" s="5"/>
+      <c r="K29" s="5" t="s">
+        <v>240</v>
+      </c>
       <c r="L29" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M29" s="6"/>
+        <v>209</v>
+      </c>
+      <c r="M29" s="6" t="s">
+        <v>242</v>
+      </c>
     </row>
     <row r="30" spans="1:13" ht="22.65" customHeight="1">
       <c r="A30" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="C30" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="B30" s="5" t="s">
+      <c r="D30" s="5" t="s">
         <v>199</v>
       </c>
-      <c r="C30" s="5" t="s">
+      <c r="E30" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="F30" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="G30" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="H30" s="5" t="s">
         <v>200</v>
       </c>
-      <c r="D30" s="5" t="s">
+      <c r="I30" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="E30" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="F30" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="G30" s="5" t="s">
-        <v>145</v>
-      </c>
-      <c r="H30" s="5" t="s">
+      <c r="J30" s="5" t="s">
         <v>202</v>
       </c>
-      <c r="I30" s="5" t="s">
-        <v>203</v>
-      </c>
-      <c r="J30" s="5" t="s">
-        <v>204</v>
-      </c>
-      <c r="K30" s="5"/>
+      <c r="K30" s="5" t="s">
+        <v>234</v>
+      </c>
       <c r="L30" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M30" s="6"/>
+        <v>209</v>
+      </c>
+      <c r="M30" s="6" t="s">
+        <v>242</v>
+      </c>
     </row>
     <row r="31" spans="1:13" ht="22.65" customHeight="1">
       <c r="A31" s="7" t="s">
+        <v>203</v>
+      </c>
+      <c r="B31" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="C31" s="8" t="s">
+        <v>204</v>
+      </c>
+      <c r="D31" s="8" t="s">
         <v>205</v>
       </c>
-      <c r="B31" s="8" t="s">
-        <v>130</v>
-      </c>
-      <c r="C31" s="8" t="s">
+      <c r="E31" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="F31" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="G31" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="H31" s="8" t="s">
         <v>206</v>
       </c>
-      <c r="D31" s="8" t="s">
+      <c r="I31" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="J31" s="8" t="s">
         <v>207</v>
       </c>
-      <c r="E31" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="F31" s="8" t="s">
-        <v>130</v>
-      </c>
-      <c r="G31" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="H31" s="8" t="s">
-        <v>208</v>
-      </c>
-      <c r="I31" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="J31" s="8" t="s">
-        <v>209</v>
-      </c>
-      <c r="K31" s="8"/>
-      <c r="L31" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="M31" s="9"/>
+      <c r="K31" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="L31" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="M31" s="6" t="s">
+        <v>242</v>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation type="list" sqref="L2:L31" xr:uid="{14F475B6-7B2E-451D-ADBF-472859C086F6}">
+    <dataValidation type="list" sqref="L28:L31" xr:uid="{14F475B6-7B2E-451D-ADBF-472859C086F6}">
       <formula1>"Not Executed,Pass,Fail,Blocked"</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="F2:F31" xr:uid="{4DAAB17B-E3A8-4B95-B6CB-0DB32ABACA09}">

</xml_diff>